<commit_message>
fix(pipeline): resolve meta spend zeroing and missing utm mapping for attribution
</commit_message>
<xml_diff>
--- a/output/satyam_7d.xlsx
+++ b/output/satyam_7d.xlsx
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3795</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="14">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3712</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="15">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>97.8129117259552</v>
+        <v>98.00976342470898</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.187088274044796</v>
+        <v>1.990236575291025</v>
       </c>
     </row>
     <row r="18">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3715</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="19">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
@@ -1584,7 +1584,7 @@
   <dimension ref="A1:AB71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -1757,8 +1757,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>46242</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -1854,8 +1856,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>46242</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1951,8 +1955,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>46242</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2048,8 +2054,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>46242</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -2145,8 +2153,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>46242</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -2242,8 +2252,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>46242</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -2339,8 +2351,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>46242</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -2436,8 +2450,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>46242</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -2533,8 +2549,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>46242</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -2630,8 +2648,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>46242</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -2727,8 +2747,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
-        <v>46242</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -2824,8 +2846,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>46242</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2921,8 +2945,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>46242</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -3018,8 +3044,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>46242</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -3115,8 +3143,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>46242</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -3212,8 +3242,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>46242</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3309,8 +3341,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>46242</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -3406,8 +3440,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>46242</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -3503,8 +3539,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>46242</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -3600,8 +3638,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>46242</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -3697,8 +3737,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>46242</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -3794,8 +3836,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>46242</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -3896,8 +3940,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
-        <v>46242</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -3993,8 +4039,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>46242</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -4090,8 +4138,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>46242</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -4192,8 +4242,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>46242</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -4289,8 +4341,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>46242</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -4386,8 +4440,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>46242</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -4483,8 +4539,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>46242</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -4580,8 +4638,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>46242</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -4677,8 +4737,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
-        <v>46242</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -4774,8 +4836,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>46242</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -4871,8 +4935,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>46242</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -4968,8 +5034,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
-        <v>46242</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -5065,8 +5133,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
-        <v>46242</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -5162,8 +5232,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
-        <v>46242</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -5259,8 +5331,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
-        <v>46242</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -5356,8 +5430,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
-        <v>46242</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -5453,8 +5529,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
-        <v>46242</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -5550,8 +5628,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>46242</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -5647,8 +5727,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
-        <v>46242</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -5744,8 +5826,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>46242</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -5841,8 +5925,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
-        <v>46242</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -5938,8 +6024,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
-        <v>46242</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -6035,8 +6123,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
-        <v>46242</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -6132,8 +6222,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
-        <v>46242</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -6229,8 +6321,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
-        <v>46242</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -6326,8 +6420,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
-        <v>46242</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -6423,8 +6519,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n">
-        <v>46242</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -6520,8 +6618,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="n">
-        <v>46242</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -6617,8 +6717,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n">
-        <v>46242</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -6714,8 +6816,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="n">
-        <v>46242</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -6811,8 +6915,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n">
-        <v>46242</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -6908,8 +7014,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="n">
-        <v>46242</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -7005,8 +7113,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="n">
-        <v>46242</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -7102,8 +7212,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="n">
-        <v>46242</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -7199,8 +7311,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n">
-        <v>46242</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -7296,8 +7410,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="n">
-        <v>46242</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -7393,8 +7509,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="n">
-        <v>46242</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -7490,8 +7608,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n">
-        <v>46242</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -7587,8 +7707,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="n">
-        <v>46242</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -7684,8 +7806,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n">
-        <v>46242</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -7781,8 +7905,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
-        <v>46242</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -7878,8 +8004,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
-        <v>46242</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -7975,8 +8103,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n">
-        <v>46242</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -8072,8 +8202,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n">
-        <v>46242</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -8169,8 +8301,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="n">
-        <v>46242</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -8266,8 +8400,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="n">
-        <v>46242</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -8363,8 +8499,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="n">
-        <v>46242</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -8460,8 +8598,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="n">
-        <v>46242</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -8810,10 +8950,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3795</v>
+        <v>2663</v>
       </c>
       <c r="D9" t="n">
-        <v>3795</v>
+        <v>2663</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -15398,16 +15538,16 @@
         <v>231716.54</v>
       </c>
       <c r="D2" t="n">
-        <v>1992</v>
+        <v>1367</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>169.5073445501097</v>
       </c>
       <c r="F2" t="n">
         <v>28</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1.405622489959839</v>
+        <v>2.04828090709583</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>251972</v>
@@ -15445,7 +15585,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>732</v>
+        <v>534</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
@@ -15454,7 +15594,7 @@
         <v>9</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1.229508196721312</v>
+        <v>1.685393258426966</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>80991</v>
@@ -15498,16 +15638,16 @@
         <v>50404.05</v>
       </c>
       <c r="D4" t="n">
-        <v>598</v>
+        <v>397</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>126.9623425692695</v>
       </c>
       <c r="F4" t="n">
         <v>5</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.8361204013377926</v>
+        <v>1.259445843828715</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>44995</v>
@@ -15545,7 +15685,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>243</v>
+        <v>211</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -15554,7 +15694,7 @@
         <v>4</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1.646090534979424</v>
+        <v>1.895734597156398</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>35996</v>
@@ -15598,7 +15738,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
@@ -15607,7 +15747,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3.448275862068965</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>8999</v>
@@ -15651,7 +15791,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -15660,7 +15800,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1.666666666666667</v>
+        <v>3.125</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>8999</v>
@@ -15704,16 +15844,20 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="4" t="n">
-        <v>5.555555555555555</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H8" s="2" t="n">
         <v>8999</v>
@@ -19674,7 +19818,7 @@
         <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>0</v>
@@ -19723,7 +19867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -19823,7 +19967,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -19832,7 +19976,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3.448275862068965</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>8999</v>
@@ -20035,16 +20179,16 @@
         <v>118068.4177208835</v>
       </c>
       <c r="D6" t="n">
-        <v>1015</v>
+        <v>691</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>170.8660169622048</v>
       </c>
       <c r="F6" t="n">
         <v>13</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1.280788177339901</v>
+        <v>1.881331403762663</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>116987</v>
@@ -20082,16 +20226,16 @@
         <v>22334.1243373494</v>
       </c>
       <c r="D7" t="n">
-        <v>192</v>
+        <v>124</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>180.1139059463661</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2.604166666666667</v>
+        <v>4.032258064516129</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>44995</v>
@@ -20129,16 +20273,16 @@
         <v>56765.89935742972</v>
       </c>
       <c r="D8" t="n">
-        <v>488</v>
+        <v>337</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>168.444805214925</v>
       </c>
       <c r="F8" t="n">
         <v>8</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>1.639344262295082</v>
+        <v>2.373887240356083</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>71992</v>
@@ -20176,16 +20320,16 @@
         <v>34548.09858433735</v>
       </c>
       <c r="D9" t="n">
-        <v>297</v>
+        <v>215</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>160.6888306248249</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.6734006734006733</v>
+        <v>0.9302325581395349</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>17998</v>
@@ -20223,10 +20367,10 @@
         <v>842.8770903010034</v>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>84.28770903010033</v>
+        <v>210.7192725752508</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -20272,16 +20416,16 @@
         <v>49561.172909699</v>
       </c>
       <c r="D11" t="n">
-        <v>588</v>
+        <v>393</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>126.1098547320585</v>
       </c>
       <c r="F11" t="n">
         <v>5</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.8503401360544218</v>
+        <v>1.272264631043257</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>44995</v>
@@ -20319,7 +20463,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>288</v>
+        <v>209</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
@@ -20328,7 +20472,7 @@
         <v>3</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.041666666666667</v>
+        <v>1.435406698564593</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>26997</v>
@@ -20372,7 +20516,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>444</v>
+        <v>325</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>0</v>
@@ -20381,7 +20525,7 @@
         <v>6</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1.351351351351351</v>
+        <v>1.846153846153846</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>53994</v>
@@ -20425,7 +20569,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>0</v>
@@ -20478,7 +20622,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -20531,7 +20675,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -20540,7 +20684,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>4</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>8999</v>
@@ -20584,16 +20728,20 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>11</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>9.090909090909092</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H17" s="2" t="n">
         <v>8999</v>
@@ -20625,7 +20773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; core it professionals | 25 - 55</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 |</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -20637,7 +20785,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -20678,7 +20826,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 |</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; data science &amp; big data &amp; data analyst | 26 - 50 |</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -20690,7 +20838,7 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -20731,7 +20879,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; data science &amp; big data &amp; data analyst | 26 - 50 |</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 |</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -20743,7 +20891,7 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -20784,7 +20932,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 |</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; web development | 26 - 50 |</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -20796,7 +20944,7 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -20837,7 +20985,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; web development | 26 - 50 |</t>
+          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -20849,22 +20997,22 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>27</v>
+        <v>211</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0</v>
+        <v>1.895734597156398</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>35996</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>35996</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -20883,14 +21031,14 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open</t>
+          <t>{{campaign.name}} &gt; {{adset.name}}</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -20902,22 +21050,22 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>243</v>
+        <v>31</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>1.646090534979424</v>
+        <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>35996</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>35996</v>
+        <v>0</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -20935,59 +21083,6 @@
         </is>
       </c>
       <c r="M23" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>{{campaign.name}} &gt; {{adset.name}}</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="n">
-        <v>51</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -21004,7 +21099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -21104,7 +21199,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -21113,7 +21208,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3.448275862068965</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>8999</v>
@@ -21316,16 +21411,16 @@
         <v>118068.4177208835</v>
       </c>
       <c r="D6" t="n">
-        <v>1015</v>
+        <v>691</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>170.8660169622048</v>
       </c>
       <c r="F6" t="n">
         <v>13</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1.280788177339901</v>
+        <v>1.881331403762663</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>116987</v>
@@ -21363,16 +21458,16 @@
         <v>22334.1243373494</v>
       </c>
       <c r="D7" t="n">
-        <v>192</v>
+        <v>124</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>180.1139059463661</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2.604166666666667</v>
+        <v>4.032258064516129</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>44995</v>
@@ -21410,16 +21505,16 @@
         <v>28150.3025502008</v>
       </c>
       <c r="D8" t="n">
-        <v>242</v>
+        <v>171</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>164.6216523403556</v>
       </c>
       <c r="F8" t="n">
         <v>5</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>2.066115702479339</v>
+        <v>2.923976608187134</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>44995</v>
@@ -21506,16 +21601,16 @@
         <v>27452.36116465864</v>
       </c>
       <c r="D10" t="n">
-        <v>236</v>
+        <v>156</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>175.9766741324271</v>
       </c>
       <c r="F10" t="n">
         <v>3</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1.271186440677966</v>
+        <v>1.923076923076923</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>26997</v>
@@ -21602,16 +21697,16 @@
         <v>34431.77502008032</v>
       </c>
       <c r="D12" t="n">
-        <v>296</v>
+        <v>214</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>160.8961449536464</v>
       </c>
       <c r="F12" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.9345794392523363</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>17998</v>
@@ -21649,10 +21744,10 @@
         <v>842.8770903010034</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>84.28770903010033</v>
+        <v>210.7192725752508</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -21698,16 +21793,16 @@
         <v>49561.172909699</v>
       </c>
       <c r="D14" t="n">
-        <v>588</v>
+        <v>393</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>126.1098547320585</v>
       </c>
       <c r="F14" t="n">
         <v>5</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.8503401360544218</v>
+        <v>1.272264631043257</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>44995</v>
@@ -21786,7 +21881,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; it &amp; technical services &gt; foremostleads-gs-13-09- ai video &lt;0504.mp4&gt; – copy 2</t>
+          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; it &amp; technical services &gt; foremostleads-gs-13-09&lt;attention it professionals if you are an it engineer&gt; – copy</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -21798,22 +21893,22 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>208</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0</v>
+        <v>1.442307692307692</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>26997</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>26997</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -21832,14 +21927,14 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; it &amp; technical services &gt; foremostleads-gs-13-09&lt;attention it professionals if you are an it engineer&gt; – copy</t>
+          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; programming language &gt; foremost leads-13-09&lt;do you know which countries are hiring&gt; – copy 2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -21851,22 +21946,22 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>286</v>
+        <v>1</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1.048951048951049</v>
+        <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>26997</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>26997</v>
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -21885,14 +21980,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; programming language &gt; foremost leads-13-09&lt;do you know which countries are hiring&gt; – copy 2</t>
+          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; programming language &gt; foremostleads-gs-13-09&lt;do you know which countries are actively sponsoring visas&gt; – copy 2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -21904,22 +21999,22 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>324</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0</v>
+        <v>1.851851851851852</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>53994</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>53994</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -21938,14 +22033,14 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>foremost leads &lt;&gt; cbo &lt;&gt; r1 &gt; foremost leads &lt;&gt; a1&lt;&gt; programming language &gt; foremostleads-gs-13-09&lt;do you know which countries are actively sponsoring visas&gt; – copy 2</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; data science | 30 -55 &gt; split ad 4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -21957,22 +22052,22 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>443</v>
+        <v>2</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>1.354401805869075</v>
+        <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>53994</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>53994</v>
+        <v>0</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -21991,14 +22086,14 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; data science | 30 -55 &gt; split ad 10</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; information technology | 30 -55 &gt; split ad 2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -22010,7 +22105,7 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -22051,7 +22146,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; data science | 30 -55 &gt; split ad 4</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -22063,7 +22158,7 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -22104,7 +22199,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; information technology | 30 -55 &gt; split ad 1</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -22116,7 +22211,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -22157,7 +22252,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; information technology | 30 -55 &gt; split ad 2</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 7</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -22169,22 +22264,22 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -22203,14 +22298,14 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; information technology | 30 -55 &gt; split ad 3</t>
+          <t>foremost leads | cbo | 14th august &gt; cloud &amp; data professionals | 25 - 55 &gt; abhishek pal 2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -22222,22 +22317,26 @@
         <v>0</v>
       </c>
       <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>0</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -22256,14 +22355,14 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 5</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 | &gt; image ads | sticky notes | dubai's tech sector is growing fast and sponsoring visas now</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -22275,7 +22374,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -22316,7 +22415,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 6</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 | &gt; image ads | sticky notes | stop applying to places that were never going to sponsor you. find out who actually does</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -22328,7 +22427,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>0</v>
@@ -22369,7 +22468,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; software engineering | 30 -55 &gt; split ad 7</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; data science &amp; big data &amp; data analyst | 26 - 50 | &gt; image ads | whiteboard | pick the right country for your experience. not just what's trending</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -22381,22 +22480,22 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>33.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>8999</v>
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -22415,14 +22514,14 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; cloud &amp; data professionals | 25 - 55 &gt; abhishek pal 1</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 | &gt; image ads | sticky notes | germany is short on tech workers and hiring from india right now</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -22434,7 +22533,7 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -22475,7 +22574,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; cloud &amp; data professionals | 25 - 55 &gt; abhishek pal 2</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 | &gt; image ads | whiteboard | know what dutch companies look for before you apply</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -22487,22 +22586,22 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I29" s="5" t="n">
-        <v>8999</v>
+        <v>0</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -22521,14 +22620,14 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; core it professionals | 25 - 55 &gt; abhishek pal 5</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; web development | 26 - 50 | &gt; image ads | ignored vs shortlisted</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -22540,7 +22639,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>0</v>
@@ -22581,7 +22680,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 | &gt; image ads | sticky notes | dubai's tech sector is growing fast and sponsoring visas now</t>
+          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open &gt; foremostleads-gs-13-09- ai video &lt;0504(1).mp4&gt;</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -22593,22 +22692,22 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="2" t="n">
-        <v>0</v>
+        <v>26997</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>26997</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -22627,14 +22726,14 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; c++ | 26 - 50 | &gt; image ads | sticky notes | stop applying to places that were never going to sponsor you. find out who actually does</t>
+          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open &gt; foremostleads-gs-13-09- ai video &lt;0504.mp4&gt;</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -22646,22 +22745,22 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>171</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0</v>
+        <v>0.5847953216374269</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -22680,14 +22779,14 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; data science &amp; big data &amp; data analyst | 26 - 50 | &gt; image ads | whiteboard | pick the right country for your experience. not just what's trending</t>
+          <t>{{campaign.name}} &gt; {{adset.name}} &gt; {{ad.name}}</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -22699,7 +22798,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -22732,324 +22831,6 @@
         </is>
       </c>
       <c r="M33" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 | &gt; image ads | sticky notes | germany is short on tech workers and hiring from india right now</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" t="n">
-        <v>7</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; java &amp; java script | 26 - 50 | &gt; image ads | whiteboard | know what dutch companies look for before you apply</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; web development | 26 - 50 | &gt; image ads | ignored vs shortlisted</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>27</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open &gt; foremostleads-gs-13-09- ai video &lt;0504(1).mp4&gt;</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" t="n">
-        <v>72</v>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="n">
-        <v>3</v>
-      </c>
-      <c r="G37" s="4" t="n">
-        <v>4.166666666666666</v>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>26997</v>
-      </c>
-      <c r="I37" s="5" t="n">
-        <v>26997</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; foremostleads-gs-13-09-open &gt; foremostleads-gs-13-09- ai video &lt;0504.mp4&gt;</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>171</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0.5847953216374269</v>
-      </c>
-      <c r="H38" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I38" s="5" t="n">
-        <v>8999</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>{{campaign.name}} &gt; {{adset.name}} &gt; {{ad.name}}</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="n">
-        <v>51</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -23066,13 +22847,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -23166,7 +22947,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -23175,7 +22956,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3.448275862068965</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>8999</v>
@@ -23427,10 +23208,10 @@
         <v>465.2942570281124</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>232.6471285140562</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -23476,10 +23257,10 @@
         <v>3955.001184738956</v>
       </c>
       <c r="D8" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>164.7917160307898</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -23525,16 +23306,16 @@
         <v>12446.62137550201</v>
       </c>
       <c r="D9" t="n">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>159.5720689166924</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1.869158878504673</v>
+        <v>2.564102564102564</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>17998</v>
@@ -23572,10 +23353,10 @@
         <v>697.9413855421687</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>232.6471285140562</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -23621,16 +23402,16 @@
         <v>25940.15482931727</v>
       </c>
       <c r="D11" t="n">
-        <v>223</v>
+        <v>140</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>185.2868202094091</v>
       </c>
       <c r="F11" t="n">
         <v>3</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1.345291479820628</v>
+        <v>2.142857142857143</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>26997</v>
@@ -23668,16 +23449,16 @@
         <v>170297.6980722892</v>
       </c>
       <c r="D12" t="n">
-        <v>1464</v>
+        <v>1017</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>167.45103055289</v>
       </c>
       <c r="F12" t="n">
         <v>22</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.502732240437158</v>
+        <v>2.16322517207473</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>197978</v>
@@ -23715,16 +23496,16 @@
         <v>14540.44553212851</v>
       </c>
       <c r="D13" t="n">
-        <v>125</v>
+        <v>82</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>177.3225064893721</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.8</v>
+        <v>1.219512195121951</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>8999</v>
@@ -23762,10 +23543,10 @@
         <v>2675.441977911647</v>
       </c>
       <c r="D14" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>157.3789398771557</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -23811,16 +23592,20 @@
         <v>232.6471285140562</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>116.3235642570281</v>
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="4" t="n">
-        <v>0</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H15" s="2" t="n">
         <v>0</v>
@@ -23909,10 +23694,10 @@
         <v>674.3016722408028</v>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>96.32881032011468</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -23958,16 +23743,16 @@
         <v>2444.34356187291</v>
       </c>
       <c r="D18" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>111.1065255396777</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3.448275862068965</v>
+        <v>4.545454545454546</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>8999</v>
@@ -24054,10 +23839,10 @@
         <v>2612.918979933111</v>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>124.4247133301481</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -24103,16 +23888,16 @@
         <v>43576.74556856188</v>
       </c>
       <c r="D21" t="n">
-        <v>517</v>
+        <v>338</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>128.9252827472245</v>
       </c>
       <c r="F21" t="n">
         <v>4</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.7736943907156674</v>
+        <v>1.183431952662722</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>35996</v>
@@ -24150,10 +23935,10 @@
         <v>758.5893812709031</v>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>126.4315635451505</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -24199,10 +23984,10 @@
         <v>168.5754180602007</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>84.28770903010034</v>
+        <v>168.5754180602007</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -24301,7 +24086,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -24310,7 +24095,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>3.333333333333333</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>8999</v>
@@ -24354,7 +24139,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>0</v>
@@ -24363,7 +24148,7 @@
         <v>3</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>1.851851851851852</v>
+        <v>2.830188679245283</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>26997</v>
@@ -24407,7 +24192,7 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>0</v>
@@ -24460,7 +24245,7 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -24469,7 +24254,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>1.01010101010101</v>
+        <v>1.282051282051282</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>8999</v>
@@ -24513,7 +24298,7 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>378</v>
+        <v>285</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
@@ -24522,7 +24307,7 @@
         <v>2</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.5291005291005291</v>
+        <v>0.7017543859649122</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>17998</v>
@@ -24566,7 +24351,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>0</v>
@@ -24619,7 +24404,7 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -24628,7 +24413,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>2.272727272727273</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>8999</v>
@@ -24713,7 +24498,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; facebook_instream_video</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; facebook_mobile_feed</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -24725,7 +24510,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -24766,7 +24551,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; facebook_mobile_feed</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; facebook_mobile_reels</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -24778,7 +24563,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -24819,7 +24604,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; facebook_mobile_reels</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_feed</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -24831,22 +24616,22 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -24865,14 +24650,14 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_feed</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_reels</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -24884,22 +24669,22 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I36" s="5" t="n">
-        <v>8999</v>
+        <v>0</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -24918,14 +24703,14 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_reels</t>
+          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_stories</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -24937,7 +24722,7 @@
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
@@ -24978,7 +24763,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 11th august 2026 &gt; instagram_stories</t>
+          <t>foremost leads | cbo | 14th august &gt; instagram_stories</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -24990,22 +24775,26 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -25024,14 +24813,14 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; facebook_instream_video</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; facebook_mobile_feed</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -25043,7 +24832,7 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
@@ -25084,7 +24873,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; facebook_mobile_reels</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; facebook_mobile_reels</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -25096,7 +24885,7 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
@@ -25137,7 +24926,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; instagram_feed</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_feed</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -25149,7 +24938,7 @@
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -25190,7 +24979,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; instagram_reels</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_reels</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -25202,7 +24991,7 @@
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -25243,7 +25032,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 14th august &gt; instagram_stories</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_stories</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -25255,22 +25044,22 @@
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I43" s="5" t="n">
-        <v>8999</v>
+        <v>0</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -25289,14 +25078,14 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; facebook_mobile_feed</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; others</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -25308,7 +25097,7 @@
         <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
@@ -25349,7 +25138,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; facebook_mobile_reels</t>
+          <t>foremost leads | cbo | 5th aug 2026 &gt; threads_feed</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -25361,7 +25150,7 @@
         <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>0</v>
@@ -25402,7 +25191,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_feed</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_desktop_feed</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -25414,7 +25203,7 @@
         <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0</v>
@@ -25455,7 +25244,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_reels</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_instream_video</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -25467,7 +25256,7 @@
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
@@ -25508,7 +25297,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; instagram_stories</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_mobile_feed</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -25520,7 +25309,7 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>0</v>
@@ -25561,7 +25350,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; others</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_mobile_reels</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -25573,7 +25362,7 @@
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0</v>
@@ -25614,7 +25403,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>foremost leads | cbo | 5th aug 2026 &gt; threads_feed</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_notification</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -25626,16 +25415,20 @@
         <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
-      <c r="G50" s="4" t="n">
-        <v>0</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="H50" s="2" t="n">
         <v>0</v>
@@ -25667,7 +25460,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_desktop_feed</t>
+          <t>foremostleads-gs-13-09 &gt; facebook_stories</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -25679,7 +25472,7 @@
         <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -25720,7 +25513,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_instream_video</t>
+          <t>foremostleads-gs-13-09 &gt; instagram_feed</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -25732,22 +25525,22 @@
         <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0</v>
+        <v>4.761904761904762</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I52" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -25766,14 +25559,14 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_mobile_feed</t>
+          <t>foremostleads-gs-13-09 &gt; instagram_reels</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -25785,22 +25578,22 @@
         <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>136</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>0</v>
+        <v>1.470588235294118</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>0</v>
+        <v>17998</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>17998</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -25819,14 +25612,14 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_mobile_reels</t>
+          <t>foremostleads-gs-13-09 &gt; instagram_stories</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -25838,22 +25631,22 @@
         <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="2" t="n">
-        <v>0</v>
+        <v>8999</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>8999</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -25872,14 +25665,14 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_notification</t>
+          <t>{{campaign.name}} &gt; {{placement}}</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -25891,7 +25684,7 @@
         <v>0</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -25924,271 +25717,6 @@
         </is>
       </c>
       <c r="M55" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; facebook_stories</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" t="n">
-        <v>4</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; instagram_feed</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" t="n">
-        <v>24</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" s="4" t="n">
-        <v>4.166666666666666</v>
-      </c>
-      <c r="H57" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I57" s="5" t="n">
-        <v>8999</v>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; instagram_reels</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="n">
-        <v>149</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" s="4" t="n">
-        <v>1.342281879194631</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>17998</v>
-      </c>
-      <c r="I58" s="5" t="n">
-        <v>17998</v>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>foremostleads-gs-13-09 &gt; instagram_stories</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" t="n">
-        <v>30</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" s="4" t="n">
-        <v>3.333333333333333</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>8999</v>
-      </c>
-      <c r="I59" s="5" t="n">
-        <v>8999</v>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>{{campaign.name}} &gt; {{placement}}</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" t="n">
-        <v>51</v>
-      </c>
-      <c r="E60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -26291,7 +25819,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3795</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="3">
@@ -26301,7 +25829,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3712</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="4">
@@ -26311,7 +25839,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>